<commit_message>
updated total hr calc logic
</commit_message>
<xml_diff>
--- a/test/PIPO_TEST/masterSheet_BECO.xlsx
+++ b/test/PIPO_TEST/masterSheet_BECO.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="103">
   <si>
     <t>SP No</t>
   </si>
@@ -80,9 +80,6 @@
   </si>
   <si>
     <t>DRIVER</t>
-  </si>
-  <si>
-    <t>BeDr1, BeDr2, BeDr3</t>
   </si>
   <si>
     <t>YES</t>
@@ -1810,13 +1807,13 @@
         <v>11</v>
       </c>
       <c r="E3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" t="s">
         <v>17</v>
       </c>
-      <c r="F3" t="s">
-        <v>18</v>
-      </c>
       <c r="G3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I3" s="28"/>
       <c r="J3" s="28"/>
@@ -1826,10 +1823,10 @@
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="10" t="s">
         <v>19</v>
-      </c>
-      <c r="B4" s="10" t="s">
-        <v>20</v>
       </c>
       <c r="C4" t="s">
         <v>16</v>
@@ -1838,21 +1835,21 @@
         <v>11</v>
       </c>
       <c r="E4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F4" t="s">
         <v>17</v>
       </c>
-      <c r="F4" t="s">
-        <v>18</v>
-      </c>
       <c r="G4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="10" t="s">
         <v>21</v>
-      </c>
-      <c r="B5" s="10" t="s">
-        <v>22</v>
       </c>
       <c r="C5" t="s">
         <v>16</v>
@@ -1861,21 +1858,21 @@
         <v>11</v>
       </c>
       <c r="E5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5" t="s">
         <v>17</v>
       </c>
-      <c r="F5" t="s">
-        <v>18</v>
-      </c>
       <c r="G5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="B6" s="12" t="s">
         <v>23</v>
-      </c>
-      <c r="B6" s="12" t="s">
-        <v>24</v>
       </c>
       <c r="C6" t="s">
         <v>16</v>
@@ -1884,21 +1881,21 @@
         <v>11</v>
       </c>
       <c r="E6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F6" t="s">
         <v>17</v>
       </c>
-      <c r="F6" t="s">
-        <v>18</v>
-      </c>
       <c r="G6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="B7" s="10" t="s">
         <v>25</v>
-      </c>
-      <c r="B7" s="10" t="s">
-        <v>26</v>
       </c>
       <c r="C7" t="s">
         <v>16</v>
@@ -1907,21 +1904,21 @@
         <v>11</v>
       </c>
       <c r="E7" t="s">
+        <v>12</v>
+      </c>
+      <c r="F7" t="s">
         <v>17</v>
       </c>
-      <c r="F7" t="s">
-        <v>18</v>
-      </c>
       <c r="G7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="B8" s="10" t="s">
         <v>27</v>
-      </c>
-      <c r="B8" s="10" t="s">
-        <v>28</v>
       </c>
       <c r="C8" t="s">
         <v>16</v>
@@ -1930,24 +1927,24 @@
         <v>11</v>
       </c>
       <c r="E8" t="s">
+        <v>12</v>
+      </c>
+      <c r="F8" t="s">
         <v>17</v>
       </c>
-      <c r="F8" t="s">
-        <v>18</v>
-      </c>
       <c r="G8" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9" spans="1:7">
       <c r="A9" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="B9" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="B9" s="10" t="s">
+      <c r="C9" t="s">
         <v>30</v>
-      </c>
-      <c r="C9" t="s">
-        <v>31</v>
       </c>
       <c r="D9" s="8" t="s">
         <v>11</v>
@@ -1964,13 +1961,13 @@
     </row>
     <row r="10" spans="1:7">
       <c r="A10" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B10" s="13" t="s">
         <v>32</v>
       </c>
-      <c r="B10" s="13" t="s">
+      <c r="C10" t="s">
         <v>33</v>
-      </c>
-      <c r="C10" t="s">
-        <v>34</v>
       </c>
       <c r="D10" s="8" t="s">
         <v>11</v>
@@ -1987,13 +1984,13 @@
     </row>
     <row r="11" spans="1:7">
       <c r="A11" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="B11" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="B11" s="10" t="s">
+      <c r="C11" t="s">
         <v>36</v>
-      </c>
-      <c r="C11" t="s">
-        <v>37</v>
       </c>
       <c r="D11" s="8" t="s">
         <v>11</v>
@@ -2010,13 +2007,13 @@
     </row>
     <row r="12" spans="1:7">
       <c r="A12" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="B12" s="14" t="s">
         <v>38</v>
       </c>
-      <c r="B12" s="14" t="s">
-        <v>39</v>
-      </c>
       <c r="C12" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D12" s="8" t="s">
         <v>11</v>
@@ -2033,13 +2030,13 @@
     </row>
     <row r="13" spans="1:7">
       <c r="A13" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="B13" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="B13" s="14" t="s">
+      <c r="C13" t="s">
         <v>41</v>
-      </c>
-      <c r="C13" t="s">
-        <v>42</v>
       </c>
       <c r="D13" s="8" t="s">
         <v>11</v>
@@ -2056,13 +2053,13 @@
     </row>
     <row r="14" spans="1:7">
       <c r="A14" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="B14" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="B14" s="14" t="s">
-        <v>44</v>
-      </c>
       <c r="C14" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D14" s="8" t="s">
         <v>11</v>
@@ -2079,16 +2076,16 @@
     </row>
     <row r="15" spans="1:7">
       <c r="A15" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="B15" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="B15" s="15" t="s">
+      <c r="C15" t="s">
+        <v>41</v>
+      </c>
+      <c r="D15" s="8" t="s">
         <v>46</v>
-      </c>
-      <c r="C15" t="s">
-        <v>42</v>
-      </c>
-      <c r="D15" s="8" t="s">
-        <v>47</v>
       </c>
       <c r="E15" t="s">
         <v>12</v>
@@ -2102,16 +2099,16 @@
     </row>
     <row r="16" spans="1:7">
       <c r="A16" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="B16" s="16" t="s">
         <v>48</v>
       </c>
-      <c r="B16" s="16" t="s">
-        <v>49</v>
-      </c>
       <c r="C16" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E16" t="s">
         <v>12</v>
@@ -2125,16 +2122,16 @@
     </row>
     <row r="17" spans="1:7">
       <c r="A17" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="B17" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="B17" s="16" t="s">
+      <c r="C17" t="s">
         <v>51</v>
       </c>
-      <c r="C17" t="s">
-        <v>52</v>
-      </c>
       <c r="D17" s="8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E17" t="s">
         <v>12</v>
@@ -2148,16 +2145,16 @@
     </row>
     <row r="18" spans="1:7">
       <c r="A18" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="B18" s="16" t="s">
         <v>53</v>
       </c>
-      <c r="B18" s="16" t="s">
-        <v>54</v>
-      </c>
       <c r="C18" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E18" t="s">
         <v>12</v>
@@ -2171,16 +2168,16 @@
     </row>
     <row r="19" spans="1:7">
       <c r="A19" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="B19" s="17" t="s">
         <v>55</v>
       </c>
-      <c r="B19" s="17" t="s">
-        <v>56</v>
-      </c>
       <c r="C19" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D19" s="8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E19" t="s">
         <v>12</v>
@@ -2194,16 +2191,16 @@
     </row>
     <row r="20" spans="1:7">
       <c r="A20" s="18" t="s">
+        <v>56</v>
+      </c>
+      <c r="B20" s="19" t="s">
         <v>57</v>
       </c>
-      <c r="B20" s="19" t="s">
-        <v>58</v>
-      </c>
       <c r="C20" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E20" t="s">
         <v>12</v>
@@ -2217,16 +2214,16 @@
     </row>
     <row r="21" spans="1:7">
       <c r="A21" s="20" t="s">
+        <v>58</v>
+      </c>
+      <c r="B21" s="21" t="s">
         <v>59</v>
       </c>
-      <c r="B21" s="21" t="s">
+      <c r="C21" t="s">
+        <v>41</v>
+      </c>
+      <c r="D21" s="8" t="s">
         <v>60</v>
-      </c>
-      <c r="C21" t="s">
-        <v>42</v>
-      </c>
-      <c r="D21" s="8" t="s">
-        <v>61</v>
       </c>
       <c r="E21" t="s">
         <v>12</v>
@@ -2240,16 +2237,16 @@
     </row>
     <row r="22" spans="1:7">
       <c r="A22" s="20" t="s">
+        <v>61</v>
+      </c>
+      <c r="B22" s="21" t="s">
         <v>62</v>
       </c>
-      <c r="B22" s="21" t="s">
+      <c r="C22" t="s">
         <v>63</v>
       </c>
-      <c r="C22" t="s">
-        <v>64</v>
-      </c>
       <c r="D22" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E22" t="s">
         <v>12</v>
@@ -2263,16 +2260,16 @@
     </row>
     <row r="23" spans="1:7">
       <c r="A23" s="20" t="s">
+        <v>64</v>
+      </c>
+      <c r="B23" s="22" t="s">
         <v>65</v>
       </c>
-      <c r="B23" s="22" t="s">
+      <c r="C23" t="s">
         <v>66</v>
       </c>
-      <c r="C23" t="s">
-        <v>67</v>
-      </c>
       <c r="D23" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E23" t="s">
         <v>12</v>
@@ -2286,16 +2283,16 @@
     </row>
     <row r="24" spans="1:7">
       <c r="A24" s="20" t="s">
+        <v>67</v>
+      </c>
+      <c r="B24" s="23" t="s">
         <v>68</v>
       </c>
-      <c r="B24" s="23" t="s">
+      <c r="C24" t="s">
         <v>69</v>
       </c>
-      <c r="C24" t="s">
-        <v>70</v>
-      </c>
       <c r="D24" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E24" t="s">
         <v>12</v>
@@ -2309,16 +2306,16 @@
     </row>
     <row r="25" spans="1:7">
       <c r="A25" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="B25" s="24" t="s">
         <v>71</v>
       </c>
-      <c r="B25" s="24" t="s">
-        <v>72</v>
-      </c>
       <c r="C25" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D25" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E25" t="s">
         <v>12</v>
@@ -2332,16 +2329,16 @@
     </row>
     <row r="26" spans="1:7">
       <c r="A26" s="20" t="s">
+        <v>72</v>
+      </c>
+      <c r="B26" s="25" t="s">
         <v>73</v>
       </c>
-      <c r="B26" s="25" t="s">
-        <v>74</v>
-      </c>
       <c r="C26" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D26" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E26" t="s">
         <v>12</v>
@@ -2355,16 +2352,16 @@
     </row>
     <row r="27" spans="1:7">
       <c r="A27" s="20" t="s">
+        <v>74</v>
+      </c>
+      <c r="B27" s="25" t="s">
         <v>75</v>
       </c>
-      <c r="B27" s="25" t="s">
-        <v>76</v>
-      </c>
       <c r="C27" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D27" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E27" t="s">
         <v>12</v>
@@ -2378,16 +2375,16 @@
     </row>
     <row r="28" spans="1:7">
       <c r="A28" s="20" t="s">
+        <v>76</v>
+      </c>
+      <c r="B28" s="26" t="s">
         <v>77</v>
       </c>
-      <c r="B28" s="26" t="s">
-        <v>78</v>
-      </c>
       <c r="C28" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D28" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E28" t="s">
         <v>12</v>
@@ -2401,16 +2398,16 @@
     </row>
     <row r="29" spans="1:7">
       <c r="A29" s="20" t="s">
+        <v>78</v>
+      </c>
+      <c r="B29" s="26" t="s">
         <v>79</v>
       </c>
-      <c r="B29" s="26" t="s">
-        <v>80</v>
-      </c>
       <c r="C29" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D29" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E29" t="s">
         <v>12</v>
@@ -2424,16 +2421,16 @@
     </row>
     <row r="30" spans="1:7">
       <c r="A30" s="20" t="s">
+        <v>80</v>
+      </c>
+      <c r="B30" s="27" t="s">
         <v>81</v>
       </c>
-      <c r="B30" s="27" t="s">
-        <v>82</v>
-      </c>
       <c r="C30" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D30" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E30" t="s">
         <v>12</v>
@@ -2447,16 +2444,16 @@
     </row>
     <row r="31" spans="1:7">
       <c r="A31" s="20" t="s">
+        <v>82</v>
+      </c>
+      <c r="B31" s="27" t="s">
         <v>83</v>
       </c>
-      <c r="B31" s="27" t="s">
-        <v>84</v>
-      </c>
       <c r="C31" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D31" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E31" t="s">
         <v>12</v>
@@ -2470,16 +2467,16 @@
     </row>
     <row r="32" spans="1:7">
       <c r="A32" s="20" t="s">
+        <v>84</v>
+      </c>
+      <c r="B32" s="25" t="s">
         <v>85</v>
       </c>
-      <c r="B32" s="25" t="s">
-        <v>86</v>
-      </c>
       <c r="C32" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D32" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E32" t="s">
         <v>12</v>
@@ -2493,16 +2490,16 @@
     </row>
     <row r="33" spans="1:7">
       <c r="A33" s="20" t="s">
+        <v>86</v>
+      </c>
+      <c r="B33" s="25" t="s">
         <v>87</v>
       </c>
-      <c r="B33" s="25" t="s">
-        <v>88</v>
-      </c>
       <c r="C33" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D33" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E33" t="s">
         <v>12</v>
@@ -2516,16 +2513,16 @@
     </row>
     <row r="34" spans="1:7">
       <c r="A34" s="20" t="s">
+        <v>88</v>
+      </c>
+      <c r="B34" s="25" t="s">
         <v>89</v>
       </c>
-      <c r="B34" s="25" t="s">
-        <v>90</v>
-      </c>
       <c r="C34" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D34" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E34" t="s">
         <v>12</v>
@@ -2539,16 +2536,16 @@
     </row>
     <row r="35" spans="1:7">
       <c r="A35" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="B35" s="22" t="s">
         <v>91</v>
       </c>
-      <c r="B35" s="22" t="s">
-        <v>92</v>
-      </c>
       <c r="C35" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D35" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E35" t="s">
         <v>12</v>
@@ -2580,18 +2577,18 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>94</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B2" s="3">
         <v>0.25</v>
@@ -2602,7 +2599,7 @@
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B3" s="3">
         <v>0.583333333333333</v>
@@ -2613,7 +2610,7 @@
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B4" s="3">
         <v>0.916666666666667</v>
@@ -2624,7 +2621,7 @@
     </row>
     <row r="5" spans="1:3">
       <c r="A5" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B5" s="3">
         <v>0.354166666666667</v>
@@ -2635,7 +2632,7 @@
     </row>
     <row r="6" spans="1:3">
       <c r="A6" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B6" s="3">
         <v>0.333333333333333</v>
@@ -2646,7 +2643,7 @@
     </row>
     <row r="7" spans="1:3">
       <c r="A7" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B7" s="3">
         <v>0.25</v>
@@ -2657,7 +2654,7 @@
     </row>
     <row r="8" spans="1:3">
       <c r="A8" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B8" s="3">
         <v>0.333333333333333</v>
@@ -2668,7 +2665,7 @@
     </row>
     <row r="9" spans="1:3">
       <c r="A9" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B9" s="3">
         <v>0.791666666666667</v>

</xml_diff>